<commit_message>
Add SeachParams class for URL configuration and update fetch_cidm_groups endpoint to use it for constructing search URLs
</commit_message>
<xml_diff>
--- a/oracle_postgresql_mappings.xlsx
+++ b/oracle_postgresql_mappings.xlsx
@@ -714,7 +714,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>date</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2214,6 @@
           <t>connect_by_root</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2222,7 +2221,6 @@
           <t>sys_connect_by_path</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2230,7 +2228,6 @@
           <t>level</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2363,7 +2360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3002,6 +2999,186 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>app_error_neg_20110</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>MDM_THEME_MOLECULE_MAP_IOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>app_error_neg_20111</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">THE ADDRESS CANNOT BE UPDATED BECAUSE THE ADDRESS TYPE IS DIFFERENT. OLD ADDRESS TYPE: </t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>app_error_neg_20112</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>AN ADDRESS ALREADY EXISTS FOR THIS COMPANY AND ADDRESS TYPE. TO MODIFY THE EXISTING ADDRESS, PLEASE USE THE UPDATE BUTTON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>app_error_neg_20113</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>IT IS NOT ALLOWED TO INVALIDATE/DELETE THIS TYPE OF ADDRESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>app_error_neg_20120</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>MDM_V_THEMES_IOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>app_error_neg_20115</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>MDM_V_THEMES_IOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>app_error_neg_20116</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>MDM_V_THEMES_IOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>app_error_neg_20117</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>MDM_V_THEMES_IOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>app_error_neg_20118</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>THIS IS NOT A VALID MOLECULE ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>app_error_neg_20119</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>MDM_V_THEMES_IOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>app_error_neg_20101</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>THIS IS NOT A VALID THEME NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>app_error_neg_20400</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>THIS THEME DESCRIPTION ALREADY EXISTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>app_error_neg_20900</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>DEBUG IN THEMES IOF STANDARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Exception handler for: 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Exception handler for: 5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>